<commit_message>
Actualiza portafolio 2026-07-11 19:23 UTC
</commit_message>
<xml_diff>
--- a/data/50001473 - MAPIMI B.xlsx
+++ b/data/50001473 - MAPIMI B.xlsx
@@ -4467,7 +4467,7 @@
         <v>46204.76285167824</v>
       </c>
       <c r="D53" s="8">
-        <v>46204.76285297454</v>
+        <v>46214.35028032407</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>172</v>
@@ -4772,7 +4772,7 @@
         <v>46204.762805509265</v>
       </c>
       <c r="D58" s="5">
-        <v>46204.762806909726</v>
+        <v>46214.33568045139</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>213</v>
@@ -5203,7 +5203,7 @@
       </c>
       <c r="C65" s="9"/>
       <c r="D65" s="8">
-        <v>46204.76253861111</v>
+        <v>46214.35144533565</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>234</v>

</xml_diff>